<commit_message>
feature :- chnage add member scroll and issue fix
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="ELP_Users" sheetId="1" r:id="rId1"/>
+    <sheet name="YouthClubData" r:id="rId5" sheetId="2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,9 +28,63 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
   <si>
     <t>Email</t>
+  </si>
+  <si>
+    <t>Youth Club Name</t>
+  </si>
+  <si>
+    <t>Creator Email</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 9427</t>
+  </si>
+  <si>
+    <t>YvoneBerge@yopmail.com</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 9583</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 9842</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 7848</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 6074</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 8562</t>
+  </si>
+  <si>
+    <t>RayFlatley@yopmail.com</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 7897</t>
+  </si>
+  <si>
+    <t>ZoraidaAnderson@yopmail.com</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 9462</t>
+  </si>
+  <si>
+    <t>MrsKathaleenPrice@yopmail.com</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 5629</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 148</t>
+  </si>
+  <si>
+    <t>WilfordRutherford@yopmail.com</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 2262</t>
   </si>
 </sst>
 </file>
@@ -1002,7 +1057,7 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
     </row>
@@ -1010,4 +1065,110 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
revert: remove VO module code, keep only realistic test data changes
Reverts all VO-related code (pages, tests, suites, resources, workflow changes)
while preserving the realistic test data improvements in YouthProfilePage and BlogPage.

VO code will be re-merged via proper PR when ready for main.
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23256" windowHeight="12204"/>
+    <workbookView windowWidth="24980" windowHeight="12200"/>
   </bookViews>
   <sheets>
     <sheet name="ELP_Users" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -27,19 +27,22 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
     <t>Email</t>
-  </si>
-  <si>
-    <t>shaurya1@yopmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -47,16 +50,353 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -64,17 +404,306 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -363,27 +992,22 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feature - add testing-all-module
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="33">
   <si>
     <t>Email</t>
   </si>
@@ -124,6 +124,9 @@
   </si>
   <si>
     <t>Youth Club Automation 3470</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 1473</t>
   </si>
 </sst>
 </file>
@@ -1108,7 +1111,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1271,6 +1274,14 @@
         <v>4</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature :- changes in flow ,now 6 member login and accpect the yc
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="43">
   <si>
     <t>Email</t>
   </si>
@@ -136,6 +136,27 @@
   </si>
   <si>
     <t>Youth Club Automation 4394</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 3667</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 3909</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 7600</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 7218</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 7891</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 6389</t>
+  </si>
+  <si>
+    <t>Youth Club Automation 2517</t>
   </si>
 </sst>
 </file>
@@ -1120,7 +1141,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1307,6 +1328,62 @@
         <v>34</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="B29" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="B30" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature fix issue that randmoly coming
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="52">
   <si>
     <t>Email</t>
   </si>
@@ -181,6 +181,9 @@
   </si>
   <si>
     <t>Youth Club Automation 3456</t>
+  </si>
+  <si>
+    <t>Sankalp Enclave Elite Youth Club</t>
   </si>
 </sst>
 </file>
@@ -1165,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1472,6 +1475,14 @@
         <v>34</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
just run add data in excel
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="53">
   <si>
     <t>Email</t>
   </si>
@@ -184,6 +184,9 @@
   </si>
   <si>
     <t>Sankalp Enclave Elite Youth Club</t>
+  </si>
+  <si>
+    <t>Umang Ward Core Youth Club</t>
   </si>
 </sst>
 </file>
@@ -1168,7 +1171,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1483,6 +1486,14 @@
         <v>34</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="B40" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature :- super admin logic change and  youthclubmember excel add colmun for data tracking
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="54">
   <si>
     <t>Email</t>
   </si>
@@ -187,6 +187,9 @@
   </si>
   <si>
     <t>Umang Ward Core Youth Club</t>
+  </si>
+  <si>
+    <t>Sankalp Vihar Alpha Youth Club</t>
   </si>
 </sst>
 </file>
@@ -1171,7 +1174,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1494,6 +1497,14 @@
         <v>34</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="B41" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
featire :0 issue fix and implement unique emai id for registration member flow
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="56">
   <si>
     <t>Email</t>
   </si>
@@ -190,6 +190,12 @@
   </si>
   <si>
     <t>Sankalp Vihar Alpha Youth Club</t>
+  </si>
+  <si>
+    <t>Udaan Sector Elite Youth Club</t>
+  </si>
+  <si>
+    <t>BartonPouros@yopmail.com</t>
   </si>
 </sst>
 </file>
@@ -1174,7 +1180,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1505,6 +1511,14 @@
         <v>34</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B42" t="s" s="0">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feature :- Server (Mac): Logout might not fully clear the session, or the page loads differently with Chrome 149 on Mac - fixed
</commit_message>
<xml_diff>
--- a/resources/Partner_prod.xlsx
+++ b/resources/Partner_prod.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="57">
   <si>
     <t>Email</t>
   </si>
@@ -196,6 +196,9 @@
   </si>
   <si>
     <t>BartonPouros@yopmail.com</t>
+  </si>
+  <si>
+    <t>Prerana Colony Apex Youth Club</t>
   </si>
 </sst>
 </file>
@@ -1180,7 +1183,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1519,6 +1522,14 @@
         <v>55</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="B43" t="s" s="0">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>